<commit_message>
feat: Added a potential GUI method by wrapping IO and interrupting it
</commit_message>
<xml_diff>
--- a/examples/4_docFinalResultsLeah.xlsx
+++ b/examples/4_docFinalResultsLeah.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10916"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sammybehrooz-kafshdooz/Library/CloudStorage/GoogleDrive-sammybehrooz@gmail.com/.shortcut-targets-by-id/1HwJ_0Wuc1XstUv-KD7fSByBVSjzU7c6j/ESC Acton Staff/04_Competitions/02_House Championships/2024 Winter/Main Pool /Ryan/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ryan\Desktop\ESC\HouseChamps\examples\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B681DB17-A4EC-9A4C-804A-ED45028BC2AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A120215C-224F-4BAD-A179-8FAA7F4603AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3480" yWindow="2560" windowWidth="27640" windowHeight="16940" xr2:uid="{5647A999-F5AF-EB45-9E71-155BFC9A85A9}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" xr2:uid="{5647A999-F5AF-EB45-9E71-155BFC9A85A9}"/>
   </bookViews>
   <sheets>
     <sheet name="Finals" sheetId="1" r:id="rId1"/>
@@ -3238,6 +3238,15 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -3246,22 +3255,13 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -3603,34 +3603,34 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:I406"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11.46484375" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="7.83203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.796875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.83203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.1640625" hidden="1" customWidth="1"/>
-    <col min="5" max="5" width="5.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.1328125" hidden="1" customWidth="1"/>
+    <col min="5" max="5" width="5.1328125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="7.33203125" customWidth="1"/>
-    <col min="7" max="7" width="26.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="26.46484375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="15" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="17.6640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="7.83203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="7.796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="179" t="s">
+    <row r="1" spans="1:9" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.95">
+      <c r="A1" s="176" t="s">
         <v>639</v>
       </c>
-      <c r="B1" s="180"/>
-      <c r="C1" s="180"/>
-      <c r="D1" s="180"/>
-      <c r="E1" s="180"/>
-      <c r="F1" s="180"/>
-      <c r="G1" s="180"/>
-      <c r="H1" s="180"/>
-      <c r="I1" s="181"/>
-    </row>
-    <row r="2" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B1" s="177"/>
+      <c r="C1" s="177"/>
+      <c r="D1" s="177"/>
+      <c r="E1" s="177"/>
+      <c r="F1" s="177"/>
+      <c r="G1" s="177"/>
+      <c r="H1" s="177"/>
+      <c r="I1" s="178"/>
+    </row>
+    <row r="2" spans="1:9" ht="21" thickBot="1" x14ac:dyDescent="0.8">
       <c r="A2" s="71" t="s">
         <v>38</v>
       </c>
@@ -3659,7 +3659,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A3" s="47">
         <v>4</v>
       </c>
@@ -3688,7 +3688,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" ht="21.4" x14ac:dyDescent="0.8">
       <c r="A4" s="42">
         <v>3</v>
       </c>
@@ -3701,7 +3701,7 @@
       <c r="H4" s="169"/>
       <c r="I4" s="166"/>
     </row>
-    <row r="5" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" ht="21.4" x14ac:dyDescent="0.8">
       <c r="A5" s="42">
         <v>5</v>
       </c>
@@ -3714,7 +3714,7 @@
       <c r="H5" s="167"/>
       <c r="I5" s="166"/>
     </row>
-    <row r="6" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" ht="21.4" x14ac:dyDescent="0.8">
       <c r="A6" s="42">
         <v>2</v>
       </c>
@@ -3727,7 +3727,7 @@
       <c r="H6" s="168"/>
       <c r="I6" s="166"/>
     </row>
-    <row r="7" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" ht="21.4" x14ac:dyDescent="0.8">
       <c r="A7" s="42">
         <v>6</v>
       </c>
@@ -3740,7 +3740,7 @@
       <c r="H7" s="167"/>
       <c r="I7" s="166"/>
     </row>
-    <row r="8" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" ht="21.75" thickBot="1" x14ac:dyDescent="0.85">
       <c r="A8" s="37">
         <v>1</v>
       </c>
@@ -3753,7 +3753,7 @@
       <c r="H8" s="165"/>
       <c r="I8" s="164"/>
     </row>
-    <row r="9" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" ht="21.75" thickBot="1" x14ac:dyDescent="0.85">
       <c r="A9" s="148"/>
       <c r="B9" s="163"/>
       <c r="C9" s="163"/>
@@ -3764,20 +3764,20 @@
       <c r="H9" s="159"/>
       <c r="I9" s="158"/>
     </row>
-    <row r="10" spans="1:9" ht="27" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A10" s="176" t="s">
+    <row r="10" spans="1:9" ht="25.15" thickBot="1" x14ac:dyDescent="0.95">
+      <c r="A10" s="179" t="s">
         <v>634</v>
       </c>
-      <c r="B10" s="177"/>
-      <c r="C10" s="177"/>
-      <c r="D10" s="177"/>
-      <c r="E10" s="177"/>
-      <c r="F10" s="177"/>
-      <c r="G10" s="177"/>
-      <c r="H10" s="177"/>
-      <c r="I10" s="178"/>
-    </row>
-    <row r="11" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B10" s="180"/>
+      <c r="C10" s="180"/>
+      <c r="D10" s="180"/>
+      <c r="E10" s="180"/>
+      <c r="F10" s="180"/>
+      <c r="G10" s="180"/>
+      <c r="H10" s="180"/>
+      <c r="I10" s="181"/>
+    </row>
+    <row r="11" spans="1:9" ht="21" thickBot="1" x14ac:dyDescent="0.8">
       <c r="A11" s="71" t="s">
         <v>38</v>
       </c>
@@ -3806,7 +3806,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A12" s="157">
         <v>4</v>
       </c>
@@ -3835,7 +3835,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A13" s="154">
         <v>3</v>
       </c>
@@ -3864,7 +3864,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A14" s="154">
         <v>6</v>
       </c>
@@ -3893,7 +3893,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A15" s="154">
         <v>1</v>
       </c>
@@ -3922,7 +3922,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A16" s="154">
         <v>2</v>
       </c>
@@ -3951,7 +3951,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="17" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:9" ht="34.15" thickBot="1" x14ac:dyDescent="0.85">
       <c r="A17" s="151">
         <v>5</v>
       </c>
@@ -3980,7 +3980,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:9" ht="21.75" thickBot="1" x14ac:dyDescent="0.85">
       <c r="A18" s="148"/>
       <c r="B18" s="147"/>
       <c r="C18" s="147"/>
@@ -3991,20 +3991,20 @@
       <c r="H18" s="143"/>
       <c r="I18" s="142"/>
     </row>
-    <row r="19" spans="1:9" ht="27" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A19" s="176" t="s">
+    <row r="19" spans="1:9" ht="25.15" thickBot="1" x14ac:dyDescent="0.95">
+      <c r="A19" s="179" t="s">
         <v>617</v>
       </c>
-      <c r="B19" s="177"/>
-      <c r="C19" s="177"/>
-      <c r="D19" s="177"/>
-      <c r="E19" s="177"/>
-      <c r="F19" s="177"/>
-      <c r="G19" s="177"/>
-      <c r="H19" s="177"/>
-      <c r="I19" s="178"/>
-    </row>
-    <row r="20" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B19" s="180"/>
+      <c r="C19" s="180"/>
+      <c r="D19" s="180"/>
+      <c r="E19" s="180"/>
+      <c r="F19" s="180"/>
+      <c r="G19" s="180"/>
+      <c r="H19" s="180"/>
+      <c r="I19" s="181"/>
+    </row>
+    <row r="20" spans="1:9" ht="21" thickBot="1" x14ac:dyDescent="0.8">
       <c r="A20" s="71" t="s">
         <v>38</v>
       </c>
@@ -4033,7 +4033,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:9" ht="20.65" x14ac:dyDescent="0.75">
       <c r="A21" s="47">
         <v>3</v>
       </c>
@@ -4062,7 +4062,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:9" ht="33.4" x14ac:dyDescent="0.75">
       <c r="A22" s="42">
         <v>4</v>
       </c>
@@ -4091,7 +4091,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="23" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:9" ht="33.4" x14ac:dyDescent="0.75">
       <c r="A23" s="42">
         <v>5</v>
       </c>
@@ -4120,7 +4120,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="24" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:9" ht="33.4" x14ac:dyDescent="0.75">
       <c r="A24" s="42">
         <v>2</v>
       </c>
@@ -4149,7 +4149,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="25" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:9" ht="33.4" x14ac:dyDescent="0.75">
       <c r="A25" s="42">
         <v>6</v>
       </c>
@@ -4178,7 +4178,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="26" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:9" ht="33.75" thickBot="1" x14ac:dyDescent="0.8">
       <c r="A26" s="37">
         <v>1</v>
       </c>
@@ -4207,21 +4207,21 @@
         <v>6</v>
       </c>
     </row>
-    <row r="27" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="28" spans="1:9" ht="27" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="28" spans="1:9" ht="25.15" thickBot="1" x14ac:dyDescent="0.95">
       <c r="A28" s="97"/>
-      <c r="B28" s="177" t="s">
+      <c r="B28" s="180" t="s">
         <v>616</v>
       </c>
-      <c r="C28" s="177"/>
-      <c r="D28" s="177"/>
-      <c r="E28" s="177"/>
-      <c r="F28" s="177"/>
-      <c r="G28" s="177"/>
-      <c r="H28" s="177"/>
-      <c r="I28" s="178"/>
-    </row>
-    <row r="29" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C28" s="180"/>
+      <c r="D28" s="180"/>
+      <c r="E28" s="180"/>
+      <c r="F28" s="180"/>
+      <c r="G28" s="180"/>
+      <c r="H28" s="180"/>
+      <c r="I28" s="181"/>
+    </row>
+    <row r="29" spans="1:9" ht="21" thickBot="1" x14ac:dyDescent="0.8">
       <c r="A29" s="136" t="s">
         <v>38</v>
       </c>
@@ -4250,7 +4250,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="30" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A30" s="69">
         <v>2</v>
       </c>
@@ -4279,7 +4279,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A31" s="67">
         <v>3</v>
       </c>
@@ -4308,7 +4308,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="32" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A32" s="67">
         <v>4</v>
       </c>
@@ -4337,7 +4337,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="33" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A33" s="67">
         <v>5</v>
       </c>
@@ -4366,7 +4366,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="34" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A34" s="67">
         <v>1</v>
       </c>
@@ -4395,7 +4395,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="35" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:9" ht="34.15" thickBot="1" x14ac:dyDescent="0.85">
       <c r="A35" s="61">
         <v>6</v>
       </c>
@@ -4424,21 +4424,21 @@
         <v>6</v>
       </c>
     </row>
-    <row r="36" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="37" spans="1:9" ht="27" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="37" spans="1:9" ht="25.15" thickBot="1" x14ac:dyDescent="0.95">
       <c r="A37" s="97"/>
-      <c r="B37" s="177" t="s">
+      <c r="B37" s="180" t="s">
         <v>607</v>
       </c>
-      <c r="C37" s="177"/>
-      <c r="D37" s="177"/>
-      <c r="E37" s="177"/>
-      <c r="F37" s="177"/>
-      <c r="G37" s="177"/>
-      <c r="H37" s="177"/>
-      <c r="I37" s="178"/>
-    </row>
-    <row r="38" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C37" s="180"/>
+      <c r="D37" s="180"/>
+      <c r="E37" s="180"/>
+      <c r="F37" s="180"/>
+      <c r="G37" s="180"/>
+      <c r="H37" s="180"/>
+      <c r="I37" s="181"/>
+    </row>
+    <row r="38" spans="1:9" ht="21" thickBot="1" x14ac:dyDescent="0.8">
       <c r="A38" s="136" t="s">
         <v>38</v>
       </c>
@@ -4467,7 +4467,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="39" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A39" s="69">
         <v>4</v>
       </c>
@@ -4496,7 +4496,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A40" s="67">
         <v>3</v>
       </c>
@@ -4525,7 +4525,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="41" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A41" s="67">
         <v>5</v>
       </c>
@@ -4554,7 +4554,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="42" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A42" s="67">
         <v>2</v>
       </c>
@@ -4583,7 +4583,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="43" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A43" s="67">
         <v>6</v>
       </c>
@@ -4612,7 +4612,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="44" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:9" ht="34.15" thickBot="1" x14ac:dyDescent="0.85">
       <c r="A44" s="61">
         <v>1</v>
       </c>
@@ -4641,21 +4641,21 @@
         <v>6</v>
       </c>
     </row>
-    <row r="45" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="46" spans="1:9" ht="27" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="46" spans="1:9" ht="25.15" thickBot="1" x14ac:dyDescent="0.95">
       <c r="A46" s="97"/>
-      <c r="B46" s="177" t="s">
+      <c r="B46" s="180" t="s">
         <v>600</v>
       </c>
-      <c r="C46" s="177"/>
-      <c r="D46" s="177"/>
-      <c r="E46" s="177"/>
-      <c r="F46" s="177"/>
-      <c r="G46" s="177"/>
-      <c r="H46" s="177"/>
-      <c r="I46" s="178"/>
-    </row>
-    <row r="47" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C46" s="180"/>
+      <c r="D46" s="180"/>
+      <c r="E46" s="180"/>
+      <c r="F46" s="180"/>
+      <c r="G46" s="180"/>
+      <c r="H46" s="180"/>
+      <c r="I46" s="181"/>
+    </row>
+    <row r="47" spans="1:9" ht="21" thickBot="1" x14ac:dyDescent="0.8">
       <c r="A47" s="32" t="s">
         <v>38</v>
       </c>
@@ -4684,7 +4684,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="48" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A48" s="54">
         <v>3</v>
       </c>
@@ -4713,7 +4713,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A49" s="52">
         <v>4</v>
       </c>
@@ -4742,7 +4742,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="50" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A50" s="52">
         <v>6</v>
       </c>
@@ -4771,7 +4771,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="51" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A51" s="52">
         <v>5</v>
       </c>
@@ -4800,7 +4800,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="52" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A52" s="52">
         <v>1</v>
       </c>
@@ -4829,7 +4829,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="53" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:9" ht="34.15" thickBot="1" x14ac:dyDescent="0.85">
       <c r="A53" s="49">
         <v>2</v>
       </c>
@@ -4858,21 +4858,21 @@
         <v>6</v>
       </c>
     </row>
-    <row r="54" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="55" spans="1:9" ht="27" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="54" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="55" spans="1:9" ht="25.15" thickBot="1" x14ac:dyDescent="0.95">
       <c r="A55" s="97"/>
-      <c r="B55" s="177" t="s">
+      <c r="B55" s="180" t="s">
         <v>584</v>
       </c>
-      <c r="C55" s="177"/>
-      <c r="D55" s="177"/>
-      <c r="E55" s="177"/>
-      <c r="F55" s="177"/>
-      <c r="G55" s="177"/>
-      <c r="H55" s="177"/>
-      <c r="I55" s="178"/>
-    </row>
-    <row r="56" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C55" s="180"/>
+      <c r="D55" s="180"/>
+      <c r="E55" s="180"/>
+      <c r="F55" s="180"/>
+      <c r="G55" s="180"/>
+      <c r="H55" s="180"/>
+      <c r="I55" s="181"/>
+    </row>
+    <row r="56" spans="1:9" ht="21" thickBot="1" x14ac:dyDescent="0.8">
       <c r="A56" s="32" t="s">
         <v>38</v>
       </c>
@@ -4901,7 +4901,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="57" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A57" s="54">
         <v>4</v>
       </c>
@@ -4930,7 +4930,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="58" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A58" s="52">
         <v>3</v>
       </c>
@@ -4959,7 +4959,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="59" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A59" s="52">
         <v>5</v>
       </c>
@@ -4988,7 +4988,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="60" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:9" ht="21.4" x14ac:dyDescent="0.8">
       <c r="A60" s="52">
         <v>1</v>
       </c>
@@ -5017,7 +5017,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="61" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A61" s="52">
         <v>6</v>
       </c>
@@ -5046,7 +5046,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="62" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:9" ht="34.15" thickBot="1" x14ac:dyDescent="0.85">
       <c r="A62" s="49">
         <v>2</v>
       </c>
@@ -5075,21 +5075,21 @@
         <v>6</v>
       </c>
     </row>
-    <row r="64" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="65" spans="1:9" ht="27" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="64" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="65" spans="1:9" ht="25.15" thickBot="1" x14ac:dyDescent="0.95">
       <c r="A65" s="97"/>
-      <c r="B65" s="177" t="s">
+      <c r="B65" s="180" t="s">
         <v>573</v>
       </c>
-      <c r="C65" s="177"/>
-      <c r="D65" s="177"/>
-      <c r="E65" s="177"/>
-      <c r="F65" s="177"/>
-      <c r="G65" s="177"/>
-      <c r="H65" s="177"/>
-      <c r="I65" s="178"/>
-    </row>
-    <row r="66" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C65" s="180"/>
+      <c r="D65" s="180"/>
+      <c r="E65" s="180"/>
+      <c r="F65" s="180"/>
+      <c r="G65" s="180"/>
+      <c r="H65" s="180"/>
+      <c r="I65" s="181"/>
+    </row>
+    <row r="66" spans="1:9" ht="21" thickBot="1" x14ac:dyDescent="0.8">
       <c r="A66" s="32" t="s">
         <v>38</v>
       </c>
@@ -5118,7 +5118,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="67" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:9" ht="33" x14ac:dyDescent="0.7">
       <c r="A67" s="54">
         <v>2</v>
       </c>
@@ -5147,7 +5147,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="68" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:9" ht="33" x14ac:dyDescent="0.7">
       <c r="A68" s="52">
         <v>3</v>
       </c>
@@ -5176,7 +5176,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="69" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:9" ht="33" x14ac:dyDescent="0.7">
       <c r="A69" s="52">
         <v>4</v>
       </c>
@@ -5205,7 +5205,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="70" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:9" ht="33" x14ac:dyDescent="0.7">
       <c r="A70" s="52">
         <v>6</v>
       </c>
@@ -5234,7 +5234,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="71" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:9" ht="33" x14ac:dyDescent="0.7">
       <c r="A71" s="52">
         <v>5</v>
       </c>
@@ -5263,7 +5263,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="72" spans="1:9" ht="20" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:9" ht="33.4" thickBot="1" x14ac:dyDescent="0.75">
       <c r="A72" s="49">
         <v>1</v>
       </c>
@@ -5292,21 +5292,21 @@
         <v>6</v>
       </c>
     </row>
-    <row r="74" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="75" spans="1:9" ht="27" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="74" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="75" spans="1:9" ht="25.15" thickBot="1" x14ac:dyDescent="0.95">
       <c r="A75" s="96"/>
-      <c r="B75" s="177" t="s">
+      <c r="B75" s="180" t="s">
         <v>563</v>
       </c>
-      <c r="C75" s="177"/>
-      <c r="D75" s="177"/>
-      <c r="E75" s="177"/>
-      <c r="F75" s="177"/>
-      <c r="G75" s="177"/>
-      <c r="H75" s="177"/>
-      <c r="I75" s="178"/>
-    </row>
-    <row r="76" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C75" s="180"/>
+      <c r="D75" s="180"/>
+      <c r="E75" s="180"/>
+      <c r="F75" s="180"/>
+      <c r="G75" s="180"/>
+      <c r="H75" s="180"/>
+      <c r="I75" s="181"/>
+    </row>
+    <row r="76" spans="1:9" ht="21" thickBot="1" x14ac:dyDescent="0.8">
       <c r="A76" s="32" t="s">
         <v>38</v>
       </c>
@@ -5335,7 +5335,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="77" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:9" ht="33" x14ac:dyDescent="0.7">
       <c r="A77" s="26">
         <v>4</v>
       </c>
@@ -5364,7 +5364,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="78" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:9" ht="33" x14ac:dyDescent="0.7">
       <c r="A78" s="16">
         <v>3</v>
       </c>
@@ -5393,7 +5393,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="79" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:9" ht="33" x14ac:dyDescent="0.7">
       <c r="A79" s="16">
         <v>5</v>
       </c>
@@ -5422,7 +5422,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="80" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:9" ht="33" x14ac:dyDescent="0.7">
       <c r="A80" s="16">
         <v>2</v>
       </c>
@@ -5451,7 +5451,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="81" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:9" ht="33" x14ac:dyDescent="0.7">
       <c r="A81" s="16">
         <v>1</v>
       </c>
@@ -5480,7 +5480,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="82" spans="1:9" ht="20" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:9" ht="33.4" thickBot="1" x14ac:dyDescent="0.75">
       <c r="A82" s="8">
         <v>6</v>
       </c>
@@ -5509,21 +5509,21 @@
         <v>6</v>
       </c>
     </row>
-    <row r="83" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="84" spans="1:9" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A84" s="179" t="s">
+    <row r="83" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="84" spans="1:9" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.95">
+      <c r="A84" s="176" t="s">
         <v>549</v>
       </c>
-      <c r="B84" s="180"/>
-      <c r="C84" s="180"/>
-      <c r="D84" s="180"/>
-      <c r="E84" s="180"/>
-      <c r="F84" s="180"/>
-      <c r="G84" s="180"/>
-      <c r="H84" s="180"/>
-      <c r="I84" s="181"/>
-    </row>
-    <row r="85" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B84" s="177"/>
+      <c r="C84" s="177"/>
+      <c r="D84" s="177"/>
+      <c r="E84" s="177"/>
+      <c r="F84" s="177"/>
+      <c r="G84" s="177"/>
+      <c r="H84" s="177"/>
+      <c r="I84" s="178"/>
+    </row>
+    <row r="85" spans="1:9" ht="21" thickBot="1" x14ac:dyDescent="0.8">
       <c r="A85" s="71" t="s">
         <v>38</v>
       </c>
@@ -5552,7 +5552,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="86" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A86" s="47">
         <v>4</v>
       </c>
@@ -5581,7 +5581,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="87" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:9" ht="21.4" x14ac:dyDescent="0.8">
       <c r="A87" s="42">
         <v>3</v>
       </c>
@@ -5594,7 +5594,7 @@
       <c r="H87" s="38"/>
       <c r="I87" s="9"/>
     </row>
-    <row r="88" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:9" ht="21.4" x14ac:dyDescent="0.8">
       <c r="A88" s="42">
         <v>5</v>
       </c>
@@ -5607,7 +5607,7 @@
       <c r="H88" s="38"/>
       <c r="I88" s="9"/>
     </row>
-    <row r="89" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:9" ht="21.4" x14ac:dyDescent="0.8">
       <c r="A89" s="42">
         <v>2</v>
       </c>
@@ -5620,7 +5620,7 @@
       <c r="H89" s="50"/>
       <c r="I89" s="9"/>
     </row>
-    <row r="90" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:9" ht="21.4" x14ac:dyDescent="0.8">
       <c r="A90" s="42">
         <v>6</v>
       </c>
@@ -5633,7 +5633,7 @@
       <c r="H90" s="38"/>
       <c r="I90" s="9"/>
     </row>
-    <row r="91" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:9" ht="21.75" thickBot="1" x14ac:dyDescent="0.85">
       <c r="A91" s="37">
         <v>1</v>
       </c>
@@ -5646,21 +5646,21 @@
       <c r="H91" s="121"/>
       <c r="I91" s="1"/>
     </row>
-    <row r="92" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="93" spans="1:9" ht="27" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A93" s="176" t="s">
+    <row r="92" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="93" spans="1:9" ht="25.15" thickBot="1" x14ac:dyDescent="0.95">
+      <c r="A93" s="179" t="s">
         <v>545</v>
       </c>
-      <c r="B93" s="177"/>
-      <c r="C93" s="177"/>
-      <c r="D93" s="177"/>
-      <c r="E93" s="177"/>
-      <c r="F93" s="177"/>
-      <c r="G93" s="177"/>
-      <c r="H93" s="177"/>
-      <c r="I93" s="178"/>
-    </row>
-    <row r="94" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B93" s="180"/>
+      <c r="C93" s="180"/>
+      <c r="D93" s="180"/>
+      <c r="E93" s="180"/>
+      <c r="F93" s="180"/>
+      <c r="G93" s="180"/>
+      <c r="H93" s="180"/>
+      <c r="I93" s="181"/>
+    </row>
+    <row r="94" spans="1:9" ht="21" thickBot="1" x14ac:dyDescent="0.8">
       <c r="A94" s="71" t="s">
         <v>38</v>
       </c>
@@ -5689,7 +5689,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="95" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A95" s="47">
         <v>4</v>
       </c>
@@ -5718,7 +5718,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="96" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A96" s="42">
         <v>3</v>
       </c>
@@ -5747,7 +5747,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="97" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A97" s="42">
         <v>5</v>
       </c>
@@ -5776,7 +5776,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="98" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A98" s="42">
         <v>2</v>
       </c>
@@ -5805,7 +5805,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="99" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A99" s="42">
         <v>1</v>
       </c>
@@ -5834,7 +5834,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="100" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:9" ht="34.15" thickBot="1" x14ac:dyDescent="0.85">
       <c r="A100" s="37">
         <v>6</v>
       </c>
@@ -5863,21 +5863,21 @@
         <v>6</v>
       </c>
     </row>
-    <row r="101" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="102" spans="1:9" ht="27" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A102" s="176" t="s">
+    <row r="101" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="102" spans="1:9" ht="25.15" thickBot="1" x14ac:dyDescent="0.95">
+      <c r="A102" s="179" t="s">
         <v>531</v>
       </c>
-      <c r="B102" s="177"/>
-      <c r="C102" s="177"/>
-      <c r="D102" s="177"/>
-      <c r="E102" s="177"/>
-      <c r="F102" s="177"/>
-      <c r="G102" s="177"/>
-      <c r="H102" s="177"/>
-      <c r="I102" s="178"/>
-    </row>
-    <row r="103" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B102" s="180"/>
+      <c r="C102" s="180"/>
+      <c r="D102" s="180"/>
+      <c r="E102" s="180"/>
+      <c r="F102" s="180"/>
+      <c r="G102" s="180"/>
+      <c r="H102" s="180"/>
+      <c r="I102" s="181"/>
+    </row>
+    <row r="103" spans="1:9" ht="21" thickBot="1" x14ac:dyDescent="0.8">
       <c r="A103" s="71" t="s">
         <v>38</v>
       </c>
@@ -5906,7 +5906,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="104" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:9" ht="33.4" x14ac:dyDescent="0.75">
       <c r="A104" s="47">
         <v>4</v>
       </c>
@@ -5935,7 +5935,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="105" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:9" ht="20.65" x14ac:dyDescent="0.75">
       <c r="A105" s="42">
         <v>3</v>
       </c>
@@ -5964,7 +5964,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="106" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:9" ht="20.65" x14ac:dyDescent="0.75">
       <c r="A106" s="42">
         <v>5</v>
       </c>
@@ -5993,7 +5993,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="107" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:9" ht="33.4" x14ac:dyDescent="0.75">
       <c r="A107" s="42">
         <v>6</v>
       </c>
@@ -6022,7 +6022,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="108" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:9" ht="33.4" x14ac:dyDescent="0.75">
       <c r="A108" s="42">
         <v>2</v>
       </c>
@@ -6051,7 +6051,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="109" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:9" ht="33.75" thickBot="1" x14ac:dyDescent="0.8">
       <c r="A109" s="37">
         <v>1</v>
       </c>
@@ -6080,21 +6080,21 @@
         <v>6</v>
       </c>
     </row>
-    <row r="110" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="111" spans="1:9" ht="27" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="110" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="111" spans="1:9" ht="25.15" thickBot="1" x14ac:dyDescent="0.95">
       <c r="A111" s="96"/>
-      <c r="B111" s="183" t="s">
+      <c r="B111" s="182" t="s">
         <v>527</v>
       </c>
-      <c r="C111" s="183"/>
-      <c r="D111" s="183"/>
-      <c r="E111" s="183"/>
-      <c r="F111" s="183"/>
-      <c r="G111" s="183"/>
-      <c r="H111" s="183"/>
-      <c r="I111" s="184"/>
-    </row>
-    <row r="112" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C111" s="182"/>
+      <c r="D111" s="182"/>
+      <c r="E111" s="182"/>
+      <c r="F111" s="182"/>
+      <c r="G111" s="182"/>
+      <c r="H111" s="182"/>
+      <c r="I111" s="183"/>
+    </row>
+    <row r="112" spans="1:9" ht="21" thickBot="1" x14ac:dyDescent="0.8">
       <c r="A112" s="32" t="s">
         <v>38</v>
       </c>
@@ -6123,7 +6123,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="113" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A113" s="69">
         <v>3</v>
       </c>
@@ -6152,7 +6152,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="114" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A114" s="67">
         <v>4</v>
       </c>
@@ -6181,7 +6181,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="115" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A115" s="67">
         <v>6</v>
       </c>
@@ -6210,7 +6210,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="116" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A116" s="67">
         <v>5</v>
       </c>
@@ -6239,7 +6239,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="117" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A117" s="67">
         <v>1</v>
       </c>
@@ -6268,7 +6268,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="118" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:9" ht="34.15" thickBot="1" x14ac:dyDescent="0.85">
       <c r="A118" s="61">
         <v>2</v>
       </c>
@@ -6297,7 +6297,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="119" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A119" s="110"/>
       <c r="B119" s="110"/>
       <c r="C119" s="110"/>
@@ -6307,20 +6307,20 @@
       <c r="G119" s="110"/>
       <c r="H119" s="110"/>
     </row>
-    <row r="120" spans="1:9" ht="27" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="120" spans="1:9" ht="25.15" thickBot="1" x14ac:dyDescent="0.95">
       <c r="A120" s="96"/>
-      <c r="B120" s="183" t="s">
+      <c r="B120" s="182" t="s">
         <v>520</v>
       </c>
-      <c r="C120" s="183"/>
-      <c r="D120" s="183"/>
-      <c r="E120" s="183"/>
-      <c r="F120" s="183"/>
-      <c r="G120" s="183"/>
-      <c r="H120" s="183"/>
-      <c r="I120" s="184"/>
-    </row>
-    <row r="121" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C120" s="182"/>
+      <c r="D120" s="182"/>
+      <c r="E120" s="182"/>
+      <c r="F120" s="182"/>
+      <c r="G120" s="182"/>
+      <c r="H120" s="182"/>
+      <c r="I120" s="183"/>
+    </row>
+    <row r="121" spans="1:9" ht="21" thickBot="1" x14ac:dyDescent="0.8">
       <c r="A121" s="32" t="s">
         <v>38</v>
       </c>
@@ -6349,7 +6349,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="122" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A122" s="69">
         <v>4</v>
       </c>
@@ -6378,7 +6378,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="123" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A123" s="67">
         <v>3</v>
       </c>
@@ -6407,7 +6407,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="124" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A124" s="67">
         <v>5</v>
       </c>
@@ -6436,7 +6436,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="125" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A125" s="67">
         <v>2</v>
       </c>
@@ -6465,7 +6465,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="126" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:9" ht="29.25" x14ac:dyDescent="0.8">
       <c r="A126" s="67">
         <v>1</v>
       </c>
@@ -6494,7 +6494,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="127" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:9" ht="34.15" thickBot="1" x14ac:dyDescent="0.85">
       <c r="A127" s="61">
         <v>6</v>
       </c>
@@ -6523,21 +6523,21 @@
         <v>6</v>
       </c>
     </row>
-    <row r="128" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="129" spans="1:9" ht="27" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="128" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="129" spans="1:9" ht="25.15" thickBot="1" x14ac:dyDescent="0.95">
       <c r="A129" s="97"/>
-      <c r="B129" s="183" t="s">
+      <c r="B129" s="182" t="s">
         <v>513</v>
       </c>
-      <c r="C129" s="183"/>
-      <c r="D129" s="183"/>
-      <c r="E129" s="183"/>
-      <c r="F129" s="183"/>
-      <c r="G129" s="183"/>
-      <c r="H129" s="183"/>
-      <c r="I129" s="184"/>
-    </row>
-    <row r="130" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C129" s="182"/>
+      <c r="D129" s="182"/>
+      <c r="E129" s="182"/>
+      <c r="F129" s="182"/>
+      <c r="G129" s="182"/>
+      <c r="H129" s="182"/>
+      <c r="I129" s="183"/>
+    </row>
+    <row r="130" spans="1:9" ht="21" thickBot="1" x14ac:dyDescent="0.8">
       <c r="A130" s="32" t="s">
         <v>38</v>
       </c>
@@ -6566,7 +6566,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="131" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A131" s="54">
         <v>4</v>
       </c>
@@ -6595,7 +6595,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="132" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A132" s="52">
         <v>3</v>
       </c>
@@ -6624,7 +6624,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="133" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A133" s="52">
         <v>2</v>
       </c>
@@ -6653,7 +6653,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="134" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A134" s="52">
         <v>5</v>
       </c>
@@ -6682,7 +6682,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="135" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A135" s="52">
         <v>1</v>
       </c>
@@ -6711,7 +6711,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="136" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:9" ht="34.15" thickBot="1" x14ac:dyDescent="0.85">
       <c r="A136" s="49">
         <v>6</v>
       </c>
@@ -6740,21 +6740,21 @@
         <v>6</v>
       </c>
     </row>
-    <row r="137" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="138" spans="1:9" ht="27" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="137" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="138" spans="1:9" ht="25.15" thickBot="1" x14ac:dyDescent="0.95">
       <c r="A138" s="97"/>
-      <c r="B138" s="177" t="s">
+      <c r="B138" s="180" t="s">
         <v>503</v>
       </c>
-      <c r="C138" s="177"/>
-      <c r="D138" s="177"/>
-      <c r="E138" s="177"/>
-      <c r="F138" s="177"/>
-      <c r="G138" s="177"/>
-      <c r="H138" s="177"/>
-      <c r="I138" s="178"/>
-    </row>
-    <row r="139" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C138" s="180"/>
+      <c r="D138" s="180"/>
+      <c r="E138" s="180"/>
+      <c r="F138" s="180"/>
+      <c r="G138" s="180"/>
+      <c r="H138" s="180"/>
+      <c r="I138" s="181"/>
+    </row>
+    <row r="139" spans="1:9" ht="21" thickBot="1" x14ac:dyDescent="0.8">
       <c r="A139" s="32" t="s">
         <v>38</v>
       </c>
@@ -6783,7 +6783,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="140" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A140" s="54">
         <v>4</v>
       </c>
@@ -6812,7 +6812,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="141" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A141" s="52">
         <v>3</v>
       </c>
@@ -6841,7 +6841,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="142" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A142" s="52">
         <v>2</v>
       </c>
@@ -6870,7 +6870,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="143" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A143" s="52">
         <v>5</v>
       </c>
@@ -6899,7 +6899,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="144" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A144" s="52">
         <v>6</v>
       </c>
@@ -6928,7 +6928,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="145" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:9" ht="34.15" thickBot="1" x14ac:dyDescent="0.85">
       <c r="A145" s="49">
         <v>1</v>
       </c>
@@ -6957,21 +6957,21 @@
         <v>6</v>
       </c>
     </row>
-    <row r="146" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="147" spans="1:9" ht="27" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="146" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="147" spans="1:9" ht="25.15" thickBot="1" x14ac:dyDescent="0.95">
       <c r="A147" s="97"/>
-      <c r="B147" s="177" t="s">
+      <c r="B147" s="180" t="s">
         <v>485</v>
       </c>
-      <c r="C147" s="177"/>
-      <c r="D147" s="177"/>
-      <c r="E147" s="177"/>
-      <c r="F147" s="177"/>
-      <c r="G147" s="177"/>
-      <c r="H147" s="177"/>
-      <c r="I147" s="178"/>
-    </row>
-    <row r="148" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C147" s="180"/>
+      <c r="D147" s="180"/>
+      <c r="E147" s="180"/>
+      <c r="F147" s="180"/>
+      <c r="G147" s="180"/>
+      <c r="H147" s="180"/>
+      <c r="I147" s="181"/>
+    </row>
+    <row r="148" spans="1:9" ht="21" thickBot="1" x14ac:dyDescent="0.8">
       <c r="A148" s="32" t="s">
         <v>38</v>
       </c>
@@ -7000,7 +7000,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="149" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:9" ht="33" x14ac:dyDescent="0.7">
       <c r="A149" s="54">
         <v>4</v>
       </c>
@@ -7029,7 +7029,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="150" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:9" ht="33" x14ac:dyDescent="0.7">
       <c r="A150" s="52">
         <v>3</v>
       </c>
@@ -7058,7 +7058,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="151" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:9" ht="33" x14ac:dyDescent="0.7">
       <c r="A151" s="52">
         <v>2</v>
       </c>
@@ -7087,7 +7087,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="152" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:9" ht="33" x14ac:dyDescent="0.7">
       <c r="A152" s="52">
         <v>5</v>
       </c>
@@ -7116,7 +7116,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="153" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:9" ht="33" x14ac:dyDescent="0.7">
       <c r="A153" s="52">
         <v>6</v>
       </c>
@@ -7145,7 +7145,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="154" spans="1:9" ht="20" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:9" ht="33.4" thickBot="1" x14ac:dyDescent="0.75">
       <c r="A154" s="49">
         <v>1</v>
       </c>
@@ -7174,21 +7174,21 @@
         <v>6</v>
       </c>
     </row>
-    <row r="155" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="156" spans="1:9" ht="27" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="155" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="156" spans="1:9" ht="25.15" thickBot="1" x14ac:dyDescent="0.95">
       <c r="A156" s="96"/>
-      <c r="B156" s="177" t="s">
+      <c r="B156" s="180" t="s">
         <v>472</v>
       </c>
-      <c r="C156" s="177"/>
-      <c r="D156" s="177"/>
-      <c r="E156" s="177"/>
-      <c r="F156" s="177"/>
-      <c r="G156" s="177"/>
-      <c r="H156" s="177"/>
-      <c r="I156" s="178"/>
-    </row>
-    <row r="157" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C156" s="180"/>
+      <c r="D156" s="180"/>
+      <c r="E156" s="180"/>
+      <c r="F156" s="180"/>
+      <c r="G156" s="180"/>
+      <c r="H156" s="180"/>
+      <c r="I156" s="181"/>
+    </row>
+    <row r="157" spans="1:9" ht="21" thickBot="1" x14ac:dyDescent="0.8">
       <c r="A157" s="32" t="s">
         <v>38</v>
       </c>
@@ -7217,7 +7217,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="158" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:9" ht="33" x14ac:dyDescent="0.7">
       <c r="A158" s="26">
         <v>3</v>
       </c>
@@ -7246,7 +7246,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="159" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:9" ht="33" x14ac:dyDescent="0.7">
       <c r="A159" s="16">
         <v>2</v>
       </c>
@@ -7275,7 +7275,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="160" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:9" ht="33" x14ac:dyDescent="0.7">
       <c r="A160" s="16">
         <v>1</v>
       </c>
@@ -7304,7 +7304,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="161" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:9" ht="33" x14ac:dyDescent="0.7">
       <c r="A161" s="16">
         <v>4</v>
       </c>
@@ -7333,7 +7333,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="162" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:9" ht="33" x14ac:dyDescent="0.7">
       <c r="A162" s="16">
         <v>5</v>
       </c>
@@ -7362,7 +7362,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="163" spans="1:9" ht="20" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:9" ht="33.4" thickBot="1" x14ac:dyDescent="0.75">
       <c r="A163" s="8">
         <v>6</v>
       </c>
@@ -7391,21 +7391,21 @@
         <v>6</v>
       </c>
     </row>
-    <row r="164" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="165" spans="1:9" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A165" s="179" t="s">
+    <row r="164" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="165" spans="1:9" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.95">
+      <c r="A165" s="176" t="s">
         <v>454</v>
       </c>
-      <c r="B165" s="180"/>
-      <c r="C165" s="180"/>
-      <c r="D165" s="180"/>
-      <c r="E165" s="180"/>
-      <c r="F165" s="180"/>
-      <c r="G165" s="180"/>
-      <c r="H165" s="180"/>
-      <c r="I165" s="181"/>
-    </row>
-    <row r="166" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B165" s="177"/>
+      <c r="C165" s="177"/>
+      <c r="D165" s="177"/>
+      <c r="E165" s="177"/>
+      <c r="F165" s="177"/>
+      <c r="G165" s="177"/>
+      <c r="H165" s="177"/>
+      <c r="I165" s="178"/>
+    </row>
+    <row r="166" spans="1:9" ht="21" thickBot="1" x14ac:dyDescent="0.8">
       <c r="A166" s="71" t="s">
         <v>38</v>
       </c>
@@ -7434,7 +7434,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="167" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A167" s="47">
         <v>4</v>
       </c>
@@ -7463,7 +7463,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="168" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:9" ht="21.4" x14ac:dyDescent="0.8">
       <c r="A168" s="42">
         <v>3</v>
       </c>
@@ -7476,7 +7476,7 @@
       <c r="H168" s="38"/>
       <c r="I168" s="9"/>
     </row>
-    <row r="169" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:9" ht="21.4" x14ac:dyDescent="0.8">
       <c r="A169" s="42">
         <v>5</v>
       </c>
@@ -7489,7 +7489,7 @@
       <c r="H169" s="38"/>
       <c r="I169" s="9"/>
     </row>
-    <row r="170" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:9" ht="21.4" x14ac:dyDescent="0.8">
       <c r="A170" s="42">
         <v>2</v>
       </c>
@@ -7502,7 +7502,7 @@
       <c r="H170" s="50"/>
       <c r="I170" s="9"/>
     </row>
-    <row r="171" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:9" ht="21.4" x14ac:dyDescent="0.8">
       <c r="A171" s="42">
         <v>6</v>
       </c>
@@ -7515,7 +7515,7 @@
       <c r="H171" s="50"/>
       <c r="I171" s="9"/>
     </row>
-    <row r="172" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:9" ht="21.75" thickBot="1" x14ac:dyDescent="0.85">
       <c r="A172" s="37">
         <v>1</v>
       </c>
@@ -7528,21 +7528,21 @@
       <c r="H172" s="76"/>
       <c r="I172" s="1"/>
     </row>
-    <row r="173" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="174" spans="1:9" ht="27" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A174" s="176" t="s">
+    <row r="173" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="174" spans="1:9" ht="25.15" thickBot="1" x14ac:dyDescent="0.95">
+      <c r="A174" s="179" t="s">
         <v>449</v>
       </c>
-      <c r="B174" s="177"/>
-      <c r="C174" s="177"/>
-      <c r="D174" s="177"/>
-      <c r="E174" s="177"/>
-      <c r="F174" s="177"/>
-      <c r="G174" s="177"/>
-      <c r="H174" s="177"/>
-      <c r="I174" s="178"/>
-    </row>
-    <row r="175" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B174" s="180"/>
+      <c r="C174" s="180"/>
+      <c r="D174" s="180"/>
+      <c r="E174" s="180"/>
+      <c r="F174" s="180"/>
+      <c r="G174" s="180"/>
+      <c r="H174" s="180"/>
+      <c r="I174" s="181"/>
+    </row>
+    <row r="175" spans="1:9" ht="21" thickBot="1" x14ac:dyDescent="0.8">
       <c r="A175" s="71" t="s">
         <v>38</v>
       </c>
@@ -7571,7 +7571,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="176" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A176" s="47">
         <v>4</v>
       </c>
@@ -7600,7 +7600,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="177" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A177" s="42">
         <v>3</v>
       </c>
@@ -7629,7 +7629,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="178" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A178" s="42">
         <v>5</v>
       </c>
@@ -7658,7 +7658,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="179" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A179" s="42">
         <v>1</v>
       </c>
@@ -7687,7 +7687,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="180" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A180" s="42">
         <v>6</v>
       </c>
@@ -7716,7 +7716,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="181" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:9" ht="34.15" thickBot="1" x14ac:dyDescent="0.85">
       <c r="A181" s="37">
         <v>2</v>
       </c>
@@ -7745,21 +7745,21 @@
         <v>6</v>
       </c>
     </row>
-    <row r="182" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="183" spans="1:9" ht="27" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A183" s="176" t="s">
+    <row r="182" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="183" spans="1:9" ht="25.15" thickBot="1" x14ac:dyDescent="0.95">
+      <c r="A183" s="179" t="s">
         <v>432</v>
       </c>
-      <c r="B183" s="177"/>
-      <c r="C183" s="177"/>
-      <c r="D183" s="177"/>
-      <c r="E183" s="177"/>
-      <c r="F183" s="177"/>
-      <c r="G183" s="177"/>
-      <c r="H183" s="177"/>
-      <c r="I183" s="178"/>
-    </row>
-    <row r="184" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B183" s="180"/>
+      <c r="C183" s="180"/>
+      <c r="D183" s="180"/>
+      <c r="E183" s="180"/>
+      <c r="F183" s="180"/>
+      <c r="G183" s="180"/>
+      <c r="H183" s="180"/>
+      <c r="I183" s="181"/>
+    </row>
+    <row r="184" spans="1:9" ht="21" thickBot="1" x14ac:dyDescent="0.8">
       <c r="A184" s="71" t="s">
         <v>38</v>
       </c>
@@ -7788,7 +7788,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="185" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:9" ht="20.65" x14ac:dyDescent="0.75">
       <c r="A185" s="47">
         <v>6</v>
       </c>
@@ -7817,7 +7817,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="186" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:9" ht="33.4" x14ac:dyDescent="0.75">
       <c r="A186" s="42">
         <v>4</v>
       </c>
@@ -7846,7 +7846,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="187" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:9" ht="33.4" x14ac:dyDescent="0.75">
       <c r="A187" s="42">
         <v>3</v>
       </c>
@@ -7875,7 +7875,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="188" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:9" ht="20.65" x14ac:dyDescent="0.75">
       <c r="A188" s="42">
         <v>2</v>
       </c>
@@ -7904,7 +7904,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="189" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:9" ht="20.65" x14ac:dyDescent="0.75">
       <c r="A189" s="42">
         <v>5</v>
       </c>
@@ -7933,7 +7933,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="190" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:9" ht="33.75" thickBot="1" x14ac:dyDescent="0.8">
       <c r="A190" s="37">
         <v>1</v>
       </c>
@@ -7962,21 +7962,21 @@
         <v>6</v>
       </c>
     </row>
-    <row r="191" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="192" spans="1:9" ht="27" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="191" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="192" spans="1:9" ht="25.15" thickBot="1" x14ac:dyDescent="0.95">
       <c r="A192" s="96"/>
-      <c r="B192" s="183" t="s">
+      <c r="B192" s="182" t="s">
         <v>426</v>
       </c>
-      <c r="C192" s="183"/>
-      <c r="D192" s="183"/>
-      <c r="E192" s="183"/>
-      <c r="F192" s="183"/>
-      <c r="G192" s="183"/>
-      <c r="H192" s="183"/>
-      <c r="I192" s="184"/>
-    </row>
-    <row r="193" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C192" s="182"/>
+      <c r="D192" s="182"/>
+      <c r="E192" s="182"/>
+      <c r="F192" s="182"/>
+      <c r="G192" s="182"/>
+      <c r="H192" s="182"/>
+      <c r="I192" s="183"/>
+    </row>
+    <row r="193" spans="1:9" ht="21" thickBot="1" x14ac:dyDescent="0.8">
       <c r="A193" s="32" t="s">
         <v>38</v>
       </c>
@@ -8005,7 +8005,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="194" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A194" s="69">
         <v>4</v>
       </c>
@@ -8034,7 +8034,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="195" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A195" s="67">
         <v>3</v>
       </c>
@@ -8063,7 +8063,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="196" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A196" s="67">
         <v>5</v>
       </c>
@@ -8092,7 +8092,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="197" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A197" s="67">
         <v>1</v>
       </c>
@@ -8121,7 +8121,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="198" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A198" s="67">
         <v>2</v>
       </c>
@@ -8150,7 +8150,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="199" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:9" ht="34.15" thickBot="1" x14ac:dyDescent="0.85">
       <c r="A199" s="61">
         <v>6</v>
       </c>
@@ -8179,7 +8179,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="200" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A200" s="110"/>
       <c r="B200" s="110"/>
       <c r="C200" s="110"/>
@@ -8189,20 +8189,20 @@
       <c r="G200" s="110"/>
       <c r="H200" s="110"/>
     </row>
-    <row r="201" spans="1:9" ht="27" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="201" spans="1:9" ht="25.15" thickBot="1" x14ac:dyDescent="0.95">
       <c r="A201" s="96"/>
-      <c r="B201" s="183" t="s">
+      <c r="B201" s="182" t="s">
         <v>415</v>
       </c>
-      <c r="C201" s="183"/>
-      <c r="D201" s="183"/>
-      <c r="E201" s="183"/>
-      <c r="F201" s="183"/>
-      <c r="G201" s="183"/>
-      <c r="H201" s="183"/>
-      <c r="I201" s="184"/>
-    </row>
-    <row r="202" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C201" s="182"/>
+      <c r="D201" s="182"/>
+      <c r="E201" s="182"/>
+      <c r="F201" s="182"/>
+      <c r="G201" s="182"/>
+      <c r="H201" s="182"/>
+      <c r="I201" s="183"/>
+    </row>
+    <row r="202" spans="1:9" ht="21" thickBot="1" x14ac:dyDescent="0.8">
       <c r="A202" s="32" t="s">
         <v>38</v>
       </c>
@@ -8231,7 +8231,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="203" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A203" s="104">
         <v>4</v>
       </c>
@@ -8260,7 +8260,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="204" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A204" s="101">
         <v>3</v>
       </c>
@@ -8289,7 +8289,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="205" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A205" s="101">
         <v>5</v>
       </c>
@@ -8318,7 +8318,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="206" spans="1:9" ht="36" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A206" s="101">
         <v>2</v>
       </c>
@@ -8347,7 +8347,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="207" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A207" s="101">
         <v>6</v>
       </c>
@@ -8376,7 +8376,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="208" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:9" ht="34.15" thickBot="1" x14ac:dyDescent="0.85">
       <c r="A208" s="99">
         <v>1</v>
       </c>
@@ -8405,20 +8405,20 @@
         <v>6</v>
       </c>
     </row>
-    <row r="209" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="210" spans="1:9" ht="27" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="B210" s="182" t="s">
+    <row r="209" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="210" spans="1:9" ht="25.15" thickBot="1" x14ac:dyDescent="0.95">
+      <c r="B210" s="184" t="s">
         <v>408</v>
       </c>
-      <c r="C210" s="183"/>
-      <c r="D210" s="183"/>
-      <c r="E210" s="183"/>
-      <c r="F210" s="183"/>
-      <c r="G210" s="183"/>
-      <c r="H210" s="183"/>
-      <c r="I210" s="184"/>
-    </row>
-    <row r="211" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C210" s="182"/>
+      <c r="D210" s="182"/>
+      <c r="E210" s="182"/>
+      <c r="F210" s="182"/>
+      <c r="G210" s="182"/>
+      <c r="H210" s="182"/>
+      <c r="I210" s="183"/>
+    </row>
+    <row r="211" spans="1:9" ht="21" thickBot="1" x14ac:dyDescent="0.8">
       <c r="A211" s="32" t="s">
         <v>38</v>
       </c>
@@ -8447,7 +8447,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="212" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A212" s="54">
         <v>4</v>
       </c>
@@ -8476,7 +8476,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="213" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A213" s="52">
         <v>3</v>
       </c>
@@ -8505,7 +8505,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="214" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A214" s="52">
         <v>5</v>
       </c>
@@ -8534,7 +8534,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="215" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A215" s="52">
         <v>1</v>
       </c>
@@ -8563,7 +8563,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="216" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A216" s="52">
         <v>2</v>
       </c>
@@ -8592,7 +8592,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="217" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A217" s="52">
         <v>6</v>
       </c>
@@ -8621,21 +8621,21 @@
         <v>6</v>
       </c>
     </row>
-    <row r="218" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="219" spans="1:9" ht="27" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="218" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="219" spans="1:9" ht="25.15" thickBot="1" x14ac:dyDescent="0.95">
       <c r="A219" s="97"/>
-      <c r="B219" s="177" t="s">
+      <c r="B219" s="180" t="s">
         <v>394</v>
       </c>
-      <c r="C219" s="177"/>
-      <c r="D219" s="177"/>
-      <c r="E219" s="177"/>
-      <c r="F219" s="177"/>
-      <c r="G219" s="177"/>
-      <c r="H219" s="177"/>
-      <c r="I219" s="178"/>
-    </row>
-    <row r="220" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C219" s="180"/>
+      <c r="D219" s="180"/>
+      <c r="E219" s="180"/>
+      <c r="F219" s="180"/>
+      <c r="G219" s="180"/>
+      <c r="H219" s="180"/>
+      <c r="I219" s="181"/>
+    </row>
+    <row r="220" spans="1:9" ht="21" thickBot="1" x14ac:dyDescent="0.8">
       <c r="A220" s="32" t="s">
         <v>38</v>
       </c>
@@ -8664,7 +8664,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="221" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A221" s="54">
         <v>4</v>
       </c>
@@ -8693,7 +8693,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="222" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A222" s="52">
         <v>5</v>
       </c>
@@ -8722,7 +8722,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="223" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A223" s="52">
         <v>2</v>
       </c>
@@ -8751,7 +8751,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="224" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A224" s="52">
         <v>3</v>
       </c>
@@ -8780,7 +8780,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="225" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A225" s="52">
         <v>1</v>
       </c>
@@ -8809,7 +8809,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="226" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A226" s="52">
         <v>6</v>
       </c>
@@ -8838,21 +8838,21 @@
         <v>6</v>
       </c>
     </row>
-    <row r="227" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="228" spans="1:9" ht="27" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="227" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="228" spans="1:9" ht="25.15" thickBot="1" x14ac:dyDescent="0.95">
       <c r="A228" s="97"/>
-      <c r="B228" s="177" t="s">
+      <c r="B228" s="180" t="s">
         <v>382</v>
       </c>
-      <c r="C228" s="177"/>
-      <c r="D228" s="177"/>
-      <c r="E228" s="177"/>
-      <c r="F228" s="177"/>
-      <c r="G228" s="177"/>
-      <c r="H228" s="177"/>
-      <c r="I228" s="178"/>
-    </row>
-    <row r="229" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C228" s="180"/>
+      <c r="D228" s="180"/>
+      <c r="E228" s="180"/>
+      <c r="F228" s="180"/>
+      <c r="G228" s="180"/>
+      <c r="H228" s="180"/>
+      <c r="I228" s="181"/>
+    </row>
+    <row r="229" spans="1:9" ht="21" thickBot="1" x14ac:dyDescent="0.8">
       <c r="A229" s="32" t="s">
         <v>38</v>
       </c>
@@ -8881,7 +8881,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="230" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:9" ht="33" x14ac:dyDescent="0.7">
       <c r="A230" s="54">
         <v>3</v>
       </c>
@@ -8910,7 +8910,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="231" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:9" ht="33" x14ac:dyDescent="0.7">
       <c r="A231" s="52">
         <v>4</v>
       </c>
@@ -8939,7 +8939,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="232" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:9" ht="33" x14ac:dyDescent="0.7">
       <c r="A232" s="52">
         <v>5</v>
       </c>
@@ -8968,7 +8968,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="233" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:9" ht="33" x14ac:dyDescent="0.7">
       <c r="A233" s="52">
         <v>6</v>
       </c>
@@ -8997,7 +8997,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="234" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:9" ht="33" x14ac:dyDescent="0.7">
       <c r="A234" s="52">
         <v>1</v>
       </c>
@@ -9026,7 +9026,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="235" spans="1:9" ht="20" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:9" ht="33.4" thickBot="1" x14ac:dyDescent="0.75">
       <c r="A235" s="49">
         <v>2</v>
       </c>
@@ -9055,21 +9055,21 @@
         <v>6</v>
       </c>
     </row>
-    <row r="236" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="237" spans="1:9" ht="27" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="236" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="237" spans="1:9" ht="25.15" thickBot="1" x14ac:dyDescent="0.95">
       <c r="A237" s="96"/>
-      <c r="B237" s="177" t="s">
+      <c r="B237" s="180" t="s">
         <v>371</v>
       </c>
-      <c r="C237" s="177"/>
-      <c r="D237" s="177"/>
-      <c r="E237" s="177"/>
-      <c r="F237" s="177"/>
-      <c r="G237" s="177"/>
-      <c r="H237" s="177"/>
-      <c r="I237" s="178"/>
-    </row>
-    <row r="238" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C237" s="180"/>
+      <c r="D237" s="180"/>
+      <c r="E237" s="180"/>
+      <c r="F237" s="180"/>
+      <c r="G237" s="180"/>
+      <c r="H237" s="180"/>
+      <c r="I237" s="181"/>
+    </row>
+    <row r="238" spans="1:9" ht="21" thickBot="1" x14ac:dyDescent="0.8">
       <c r="A238" s="32" t="s">
         <v>38</v>
       </c>
@@ -9098,7 +9098,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="239" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:9" ht="33" x14ac:dyDescent="0.7">
       <c r="A239" s="54">
         <v>4</v>
       </c>
@@ -9127,7 +9127,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="240" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:9" ht="33" x14ac:dyDescent="0.7">
       <c r="A240" s="52">
         <v>3</v>
       </c>
@@ -9156,7 +9156,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="241" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:9" ht="33" x14ac:dyDescent="0.7">
       <c r="A241" s="52">
         <v>5</v>
       </c>
@@ -9185,7 +9185,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="242" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:9" ht="33" x14ac:dyDescent="0.7">
       <c r="A242" s="52">
         <v>6</v>
       </c>
@@ -9214,7 +9214,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="243" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:9" ht="33" x14ac:dyDescent="0.7">
       <c r="A243" s="52">
         <v>1</v>
       </c>
@@ -9243,7 +9243,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="244" spans="1:9" ht="20" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="244" spans="1:9" ht="33.4" thickBot="1" x14ac:dyDescent="0.75">
       <c r="A244" s="49">
         <v>2</v>
       </c>
@@ -9272,21 +9272,21 @@
         <v>6</v>
       </c>
     </row>
-    <row r="245" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="246" spans="1:9" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A246" s="179" t="s">
+    <row r="245" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="246" spans="1:9" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.95">
+      <c r="A246" s="176" t="s">
         <v>356</v>
       </c>
-      <c r="B246" s="180"/>
-      <c r="C246" s="180"/>
-      <c r="D246" s="180"/>
-      <c r="E246" s="180"/>
-      <c r="F246" s="180"/>
-      <c r="G246" s="180"/>
-      <c r="H246" s="180"/>
-      <c r="I246" s="181"/>
-    </row>
-    <row r="247" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B246" s="177"/>
+      <c r="C246" s="177"/>
+      <c r="D246" s="177"/>
+      <c r="E246" s="177"/>
+      <c r="F246" s="177"/>
+      <c r="G246" s="177"/>
+      <c r="H246" s="177"/>
+      <c r="I246" s="178"/>
+    </row>
+    <row r="247" spans="1:9" ht="21" thickBot="1" x14ac:dyDescent="0.8">
       <c r="A247" s="71" t="s">
         <v>38</v>
       </c>
@@ -9315,7 +9315,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="248" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="248" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A248" s="47">
         <v>4</v>
       </c>
@@ -9344,7 +9344,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="249" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="249" spans="1:9" ht="21.4" x14ac:dyDescent="0.8">
       <c r="A249" s="42">
         <v>3</v>
       </c>
@@ -9357,7 +9357,7 @@
       <c r="H249" s="38"/>
       <c r="I249" s="9"/>
     </row>
-    <row r="250" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="250" spans="1:9" ht="21.4" x14ac:dyDescent="0.8">
       <c r="A250" s="42">
         <v>5</v>
       </c>
@@ -9370,7 +9370,7 @@
       <c r="H250" s="50"/>
       <c r="I250" s="9"/>
     </row>
-    <row r="251" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="251" spans="1:9" ht="21.4" x14ac:dyDescent="0.8">
       <c r="A251" s="42">
         <v>2</v>
       </c>
@@ -9383,7 +9383,7 @@
       <c r="H251" s="50"/>
       <c r="I251" s="9"/>
     </row>
-    <row r="252" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="252" spans="1:9" ht="21.4" x14ac:dyDescent="0.8">
       <c r="A252" s="42">
         <v>6</v>
       </c>
@@ -9396,7 +9396,7 @@
       <c r="H252" s="50"/>
       <c r="I252" s="9"/>
     </row>
-    <row r="253" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="253" spans="1:9" ht="21.75" thickBot="1" x14ac:dyDescent="0.85">
       <c r="A253" s="37">
         <v>1</v>
       </c>
@@ -9409,21 +9409,21 @@
       <c r="H253" s="76"/>
       <c r="I253" s="1"/>
     </row>
-    <row r="254" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="255" spans="1:9" ht="27" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A255" s="176" t="s">
+    <row r="254" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="255" spans="1:9" ht="25.15" thickBot="1" x14ac:dyDescent="0.95">
+      <c r="A255" s="179" t="s">
         <v>354</v>
       </c>
-      <c r="B255" s="177"/>
-      <c r="C255" s="177"/>
-      <c r="D255" s="177"/>
-      <c r="E255" s="177"/>
-      <c r="F255" s="177"/>
-      <c r="G255" s="177"/>
-      <c r="H255" s="177"/>
-      <c r="I255" s="178"/>
-    </row>
-    <row r="256" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B255" s="180"/>
+      <c r="C255" s="180"/>
+      <c r="D255" s="180"/>
+      <c r="E255" s="180"/>
+      <c r="F255" s="180"/>
+      <c r="G255" s="180"/>
+      <c r="H255" s="180"/>
+      <c r="I255" s="181"/>
+    </row>
+    <row r="256" spans="1:9" ht="21" thickBot="1" x14ac:dyDescent="0.8">
       <c r="A256" s="71" t="s">
         <v>38</v>
       </c>
@@ -9452,7 +9452,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="257" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="257" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A257" s="47">
         <v>5</v>
       </c>
@@ -9481,7 +9481,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="258" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="258" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A258" s="42">
         <v>4</v>
       </c>
@@ -9510,7 +9510,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="259" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="259" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A259" s="42">
         <v>3</v>
       </c>
@@ -9539,7 +9539,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="260" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="260" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A260" s="42">
         <v>6</v>
       </c>
@@ -9568,7 +9568,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="261" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="261" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A261" s="42">
         <v>2</v>
       </c>
@@ -9597,7 +9597,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="262" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="262" spans="1:9" ht="34.15" thickBot="1" x14ac:dyDescent="0.85">
       <c r="A262" s="37">
         <v>1</v>
       </c>
@@ -9626,21 +9626,21 @@
         <v>6</v>
       </c>
     </row>
-    <row r="263" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="264" spans="1:9" ht="27" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A264" s="176" t="s">
+    <row r="263" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="264" spans="1:9" ht="25.15" thickBot="1" x14ac:dyDescent="0.95">
+      <c r="A264" s="179" t="s">
         <v>335</v>
       </c>
-      <c r="B264" s="177"/>
-      <c r="C264" s="177"/>
-      <c r="D264" s="177"/>
-      <c r="E264" s="177"/>
-      <c r="F264" s="177"/>
-      <c r="G264" s="177"/>
-      <c r="H264" s="177"/>
-      <c r="I264" s="178"/>
-    </row>
-    <row r="265" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B264" s="180"/>
+      <c r="C264" s="180"/>
+      <c r="D264" s="180"/>
+      <c r="E264" s="180"/>
+      <c r="F264" s="180"/>
+      <c r="G264" s="180"/>
+      <c r="H264" s="180"/>
+      <c r="I264" s="181"/>
+    </row>
+    <row r="265" spans="1:9" ht="21" thickBot="1" x14ac:dyDescent="0.8">
       <c r="A265" s="71" t="s">
         <v>38</v>
       </c>
@@ -9669,7 +9669,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="266" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="266" spans="1:9" ht="20.65" x14ac:dyDescent="0.75">
       <c r="A266" s="47">
         <v>4</v>
       </c>
@@ -9698,7 +9698,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="267" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="267" spans="1:9" ht="33.4" x14ac:dyDescent="0.75">
       <c r="A267" s="42">
         <v>3</v>
       </c>
@@ -9727,7 +9727,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="268" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="268" spans="1:9" ht="20.65" x14ac:dyDescent="0.75">
       <c r="A268" s="42">
         <v>5</v>
       </c>
@@ -9756,7 +9756,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="269" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="269" spans="1:9" ht="33.4" x14ac:dyDescent="0.75">
       <c r="A269" s="42">
         <v>2</v>
       </c>
@@ -9785,7 +9785,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="270" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="270" spans="1:9" ht="20.65" x14ac:dyDescent="0.75">
       <c r="A270" s="42">
         <v>1</v>
       </c>
@@ -9814,7 +9814,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="271" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="271" spans="1:9" ht="33.75" thickBot="1" x14ac:dyDescent="0.8">
       <c r="A271" s="37">
         <v>6</v>
       </c>
@@ -9843,21 +9843,21 @@
         <v>6</v>
       </c>
     </row>
-    <row r="272" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="273" spans="1:9" ht="27" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A273" s="176" t="s">
+    <row r="272" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="273" spans="1:9" ht="25.15" thickBot="1" x14ac:dyDescent="0.95">
+      <c r="A273" s="179" t="s">
         <v>326</v>
       </c>
-      <c r="B273" s="177"/>
-      <c r="C273" s="177"/>
-      <c r="D273" s="177"/>
-      <c r="E273" s="177"/>
-      <c r="F273" s="177"/>
-      <c r="G273" s="177"/>
-      <c r="H273" s="177"/>
-      <c r="I273" s="178"/>
-    </row>
-    <row r="274" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B273" s="180"/>
+      <c r="C273" s="180"/>
+      <c r="D273" s="180"/>
+      <c r="E273" s="180"/>
+      <c r="F273" s="180"/>
+      <c r="G273" s="180"/>
+      <c r="H273" s="180"/>
+      <c r="I273" s="181"/>
+    </row>
+    <row r="274" spans="1:9" ht="21" thickBot="1" x14ac:dyDescent="0.8">
       <c r="A274" s="71" t="s">
         <v>38</v>
       </c>
@@ -9886,7 +9886,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="275" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="275" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A275" s="69">
         <v>4</v>
       </c>
@@ -9915,7 +9915,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="276" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="276" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A276" s="67">
         <v>3</v>
       </c>
@@ -9944,7 +9944,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="277" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="277" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A277" s="67">
         <v>2</v>
       </c>
@@ -9973,7 +9973,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="278" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="278" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A278" s="67">
         <v>6</v>
       </c>
@@ -10002,7 +10002,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="279" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="279" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A279" s="67">
         <v>1</v>
       </c>
@@ -10031,7 +10031,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="280" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="280" spans="1:9" ht="34.15" thickBot="1" x14ac:dyDescent="0.85">
       <c r="A280" s="61">
         <v>5</v>
       </c>
@@ -10060,21 +10060,21 @@
         <v>6</v>
       </c>
     </row>
-    <row r="281" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="282" spans="1:9" ht="27" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A282" s="176" t="s">
+    <row r="281" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="282" spans="1:9" ht="25.15" thickBot="1" x14ac:dyDescent="0.95">
+      <c r="A282" s="179" t="s">
         <v>316</v>
       </c>
-      <c r="B282" s="177"/>
-      <c r="C282" s="177"/>
-      <c r="D282" s="177"/>
-      <c r="E282" s="177"/>
-      <c r="F282" s="177"/>
-      <c r="G282" s="177"/>
-      <c r="H282" s="177"/>
-      <c r="I282" s="178"/>
-    </row>
-    <row r="283" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B282" s="180"/>
+      <c r="C282" s="180"/>
+      <c r="D282" s="180"/>
+      <c r="E282" s="180"/>
+      <c r="F282" s="180"/>
+      <c r="G282" s="180"/>
+      <c r="H282" s="180"/>
+      <c r="I282" s="181"/>
+    </row>
+    <row r="283" spans="1:9" ht="21" thickBot="1" x14ac:dyDescent="0.8">
       <c r="A283" s="71" t="s">
         <v>38</v>
       </c>
@@ -10103,7 +10103,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="284" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="284" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A284" s="69">
         <v>3</v>
       </c>
@@ -10132,7 +10132,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="285" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="285" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A285" s="67">
         <v>4</v>
       </c>
@@ -10161,7 +10161,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="286" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="286" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A286" s="67">
         <v>2</v>
       </c>
@@ -10190,7 +10190,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="287" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="287" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A287" s="67">
         <v>5</v>
       </c>
@@ -10219,7 +10219,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="288" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="288" spans="1:9" ht="29.25" x14ac:dyDescent="0.8">
       <c r="A288" s="67">
         <v>1</v>
       </c>
@@ -10248,7 +10248,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="289" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="289" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A289" s="67">
         <v>6</v>
       </c>
@@ -10277,21 +10277,21 @@
         <v>6</v>
       </c>
     </row>
-    <row r="290" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="291" spans="1:9" ht="27" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A291" s="182" t="s">
+    <row r="290" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="291" spans="1:9" ht="25.15" thickBot="1" x14ac:dyDescent="0.95">
+      <c r="A291" s="184" t="s">
         <v>311</v>
       </c>
-      <c r="B291" s="183"/>
-      <c r="C291" s="183"/>
-      <c r="D291" s="183"/>
-      <c r="E291" s="183"/>
-      <c r="F291" s="183"/>
-      <c r="G291" s="183"/>
-      <c r="H291" s="183"/>
-      <c r="I291" s="184"/>
-    </row>
-    <row r="292" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B291" s="182"/>
+      <c r="C291" s="182"/>
+      <c r="D291" s="182"/>
+      <c r="E291" s="182"/>
+      <c r="F291" s="182"/>
+      <c r="G291" s="182"/>
+      <c r="H291" s="182"/>
+      <c r="I291" s="183"/>
+    </row>
+    <row r="292" spans="1:9" ht="21" thickBot="1" x14ac:dyDescent="0.8">
       <c r="A292" s="32" t="s">
         <v>38</v>
       </c>
@@ -10320,7 +10320,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="293" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="293" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A293" s="54">
         <v>4</v>
       </c>
@@ -10349,7 +10349,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="294" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="294" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A294" s="52">
         <v>5</v>
       </c>
@@ -10378,7 +10378,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="295" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="295" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A295" s="52">
         <v>3</v>
       </c>
@@ -10407,7 +10407,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="296" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="296" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A296" s="52">
         <v>2</v>
       </c>
@@ -10436,7 +10436,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="297" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="297" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A297" s="52">
         <v>6</v>
       </c>
@@ -10465,7 +10465,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="298" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="298" spans="1:9" ht="34.15" thickBot="1" x14ac:dyDescent="0.85">
       <c r="A298" s="49">
         <v>1</v>
       </c>
@@ -10494,21 +10494,21 @@
         <v>6</v>
       </c>
     </row>
-    <row r="299" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="300" spans="1:9" ht="27" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A300" s="176" t="s">
+    <row r="299" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="300" spans="1:9" ht="25.15" thickBot="1" x14ac:dyDescent="0.95">
+      <c r="A300" s="179" t="s">
         <v>295</v>
       </c>
-      <c r="B300" s="177"/>
-      <c r="C300" s="177"/>
-      <c r="D300" s="177"/>
-      <c r="E300" s="177"/>
-      <c r="F300" s="177"/>
-      <c r="G300" s="177"/>
-      <c r="H300" s="177"/>
-      <c r="I300" s="178"/>
-    </row>
-    <row r="301" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B300" s="180"/>
+      <c r="C300" s="180"/>
+      <c r="D300" s="180"/>
+      <c r="E300" s="180"/>
+      <c r="F300" s="180"/>
+      <c r="G300" s="180"/>
+      <c r="H300" s="180"/>
+      <c r="I300" s="181"/>
+    </row>
+    <row r="301" spans="1:9" ht="21" thickBot="1" x14ac:dyDescent="0.8">
       <c r="A301" s="32" t="s">
         <v>38</v>
       </c>
@@ -10537,7 +10537,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="302" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="302" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A302" s="54">
         <v>3</v>
       </c>
@@ -10566,7 +10566,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="303" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="303" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A303" s="52">
         <v>4</v>
       </c>
@@ -10595,7 +10595,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="304" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="304" spans="1:9" ht="21.4" x14ac:dyDescent="0.8">
       <c r="A304" s="52">
         <v>5</v>
       </c>
@@ -10624,7 +10624,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="305" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="305" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A305" s="52">
         <v>2</v>
       </c>
@@ -10653,7 +10653,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="306" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="306" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A306" s="52">
         <v>1</v>
       </c>
@@ -10682,7 +10682,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="307" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="307" spans="1:9" ht="34.15" thickBot="1" x14ac:dyDescent="0.85">
       <c r="A307" s="49">
         <v>6</v>
       </c>
@@ -10711,21 +10711,21 @@
         <v>6</v>
       </c>
     </row>
-    <row r="308" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="309" spans="1:9" ht="27" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A309" s="176" t="s">
+    <row r="308" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="309" spans="1:9" ht="25.15" thickBot="1" x14ac:dyDescent="0.95">
+      <c r="A309" s="179" t="s">
         <v>280</v>
       </c>
-      <c r="B309" s="177"/>
-      <c r="C309" s="177"/>
-      <c r="D309" s="177"/>
-      <c r="E309" s="177"/>
-      <c r="F309" s="177"/>
-      <c r="G309" s="177"/>
-      <c r="H309" s="177"/>
-      <c r="I309" s="178"/>
-    </row>
-    <row r="310" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B309" s="180"/>
+      <c r="C309" s="180"/>
+      <c r="D309" s="180"/>
+      <c r="E309" s="180"/>
+      <c r="F309" s="180"/>
+      <c r="G309" s="180"/>
+      <c r="H309" s="180"/>
+      <c r="I309" s="181"/>
+    </row>
+    <row r="310" spans="1:9" ht="21" thickBot="1" x14ac:dyDescent="0.8">
       <c r="A310" s="32" t="s">
         <v>38</v>
       </c>
@@ -10754,7 +10754,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="311" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+    <row r="311" spans="1:9" ht="33" x14ac:dyDescent="0.7">
       <c r="A311" s="26">
         <v>4</v>
       </c>
@@ -10783,7 +10783,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="312" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+    <row r="312" spans="1:9" ht="33" x14ac:dyDescent="0.7">
       <c r="A312" s="16">
         <v>3</v>
       </c>
@@ -10812,7 +10812,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="313" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+    <row r="313" spans="1:9" ht="33" x14ac:dyDescent="0.7">
       <c r="A313" s="16">
         <v>2</v>
       </c>
@@ -10841,7 +10841,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="314" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+    <row r="314" spans="1:9" ht="33" x14ac:dyDescent="0.7">
       <c r="A314" s="16">
         <v>5</v>
       </c>
@@ -10870,7 +10870,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="315" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+    <row r="315" spans="1:9" ht="33" x14ac:dyDescent="0.7">
       <c r="A315" s="16">
         <v>6</v>
       </c>
@@ -10899,7 +10899,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="316" spans="1:9" ht="20" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="316" spans="1:9" ht="33.4" thickBot="1" x14ac:dyDescent="0.75">
       <c r="A316" s="8">
         <v>1</v>
       </c>
@@ -10928,21 +10928,21 @@
         <v>40</v>
       </c>
     </row>
-    <row r="317" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="318" spans="1:9" ht="27" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A318" s="176" t="s">
+    <row r="317" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="318" spans="1:9" ht="25.15" thickBot="1" x14ac:dyDescent="0.95">
+      <c r="A318" s="179" t="s">
         <v>269</v>
       </c>
-      <c r="B318" s="177"/>
-      <c r="C318" s="177"/>
-      <c r="D318" s="177"/>
-      <c r="E318" s="177"/>
-      <c r="F318" s="177"/>
-      <c r="G318" s="177"/>
-      <c r="H318" s="177"/>
-      <c r="I318" s="178"/>
-    </row>
-    <row r="319" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B318" s="180"/>
+      <c r="C318" s="180"/>
+      <c r="D318" s="180"/>
+      <c r="E318" s="180"/>
+      <c r="F318" s="180"/>
+      <c r="G318" s="180"/>
+      <c r="H318" s="180"/>
+      <c r="I318" s="181"/>
+    </row>
+    <row r="319" spans="1:9" ht="21" thickBot="1" x14ac:dyDescent="0.8">
       <c r="A319" s="32" t="s">
         <v>38</v>
       </c>
@@ -10971,7 +10971,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="320" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+    <row r="320" spans="1:9" ht="33" x14ac:dyDescent="0.7">
       <c r="A320" s="26">
         <v>4</v>
       </c>
@@ -11000,7 +11000,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="321" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+    <row r="321" spans="1:9" ht="33" x14ac:dyDescent="0.7">
       <c r="A321" s="16">
         <v>3</v>
       </c>
@@ -11029,7 +11029,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="322" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+    <row r="322" spans="1:9" ht="33" x14ac:dyDescent="0.7">
       <c r="A322" s="16">
         <v>5</v>
       </c>
@@ -11058,7 +11058,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="323" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+    <row r="323" spans="1:9" ht="33" x14ac:dyDescent="0.7">
       <c r="A323" s="16">
         <v>2</v>
       </c>
@@ -11087,7 +11087,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="324" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+    <row r="324" spans="1:9" ht="33" x14ac:dyDescent="0.7">
       <c r="A324" s="16">
         <v>6</v>
       </c>
@@ -11116,7 +11116,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="325" spans="1:9" ht="20" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="325" spans="1:9" ht="33.4" thickBot="1" x14ac:dyDescent="0.75">
       <c r="A325" s="8">
         <v>1</v>
       </c>
@@ -11145,21 +11145,21 @@
         <v>6</v>
       </c>
     </row>
-    <row r="326" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="327" spans="1:9" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A327" s="179" t="s">
+    <row r="326" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="327" spans="1:9" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.95">
+      <c r="A327" s="176" t="s">
         <v>254</v>
       </c>
-      <c r="B327" s="180"/>
-      <c r="C327" s="180"/>
-      <c r="D327" s="180"/>
-      <c r="E327" s="180"/>
-      <c r="F327" s="180"/>
-      <c r="G327" s="180"/>
-      <c r="H327" s="180"/>
-      <c r="I327" s="181"/>
-    </row>
-    <row r="328" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B327" s="177"/>
+      <c r="C327" s="177"/>
+      <c r="D327" s="177"/>
+      <c r="E327" s="177"/>
+      <c r="F327" s="177"/>
+      <c r="G327" s="177"/>
+      <c r="H327" s="177"/>
+      <c r="I327" s="178"/>
+    </row>
+    <row r="328" spans="1:9" ht="21" thickBot="1" x14ac:dyDescent="0.8">
       <c r="A328" s="71" t="s">
         <v>38</v>
       </c>
@@ -11188,7 +11188,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="329" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="329" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A329" s="47">
         <v>4</v>
       </c>
@@ -11217,7 +11217,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="330" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="330" spans="1:9" ht="21.4" x14ac:dyDescent="0.8">
       <c r="A330" s="42">
         <v>3</v>
       </c>
@@ -11230,7 +11230,7 @@
       <c r="H330" s="38"/>
       <c r="I330" s="9"/>
     </row>
-    <row r="331" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="331" spans="1:9" ht="21.4" x14ac:dyDescent="0.8">
       <c r="A331" s="42">
         <v>5</v>
       </c>
@@ -11243,7 +11243,7 @@
       <c r="H331" s="50"/>
       <c r="I331" s="9"/>
     </row>
-    <row r="332" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="332" spans="1:9" ht="21.4" x14ac:dyDescent="0.8">
       <c r="A332" s="42">
         <v>2</v>
       </c>
@@ -11256,7 +11256,7 @@
       <c r="H332" s="50"/>
       <c r="I332" s="9"/>
     </row>
-    <row r="333" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="333" spans="1:9" ht="21.4" x14ac:dyDescent="0.8">
       <c r="A333" s="42">
         <v>6</v>
       </c>
@@ -11269,7 +11269,7 @@
       <c r="H333" s="50"/>
       <c r="I333" s="9"/>
     </row>
-    <row r="334" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="334" spans="1:9" ht="21.75" thickBot="1" x14ac:dyDescent="0.85">
       <c r="A334" s="37">
         <v>1</v>
       </c>
@@ -11282,21 +11282,21 @@
       <c r="H334" s="76"/>
       <c r="I334" s="1"/>
     </row>
-    <row r="335" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="336" spans="1:9" ht="27" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A336" s="176" t="s">
+    <row r="335" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="336" spans="1:9" ht="25.15" thickBot="1" x14ac:dyDescent="0.95">
+      <c r="A336" s="179" t="s">
         <v>248</v>
       </c>
-      <c r="B336" s="177"/>
-      <c r="C336" s="177"/>
-      <c r="D336" s="177"/>
-      <c r="E336" s="177"/>
-      <c r="F336" s="177"/>
-      <c r="G336" s="177"/>
-      <c r="H336" s="177"/>
-      <c r="I336" s="178"/>
-    </row>
-    <row r="337" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B336" s="180"/>
+      <c r="C336" s="180"/>
+      <c r="D336" s="180"/>
+      <c r="E336" s="180"/>
+      <c r="F336" s="180"/>
+      <c r="G336" s="180"/>
+      <c r="H336" s="180"/>
+      <c r="I336" s="181"/>
+    </row>
+    <row r="337" spans="1:9" ht="21" thickBot="1" x14ac:dyDescent="0.8">
       <c r="A337" s="71" t="s">
         <v>38</v>
       </c>
@@ -11325,7 +11325,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="338" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="338" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A338" s="47">
         <v>4</v>
       </c>
@@ -11354,7 +11354,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="339" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="339" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A339" s="42">
         <v>3</v>
       </c>
@@ -11383,7 +11383,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="340" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="340" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A340" s="42">
         <v>5</v>
       </c>
@@ -11412,7 +11412,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="341" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="341" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A341" s="42">
         <v>6</v>
       </c>
@@ -11441,7 +11441,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="342" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="342" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A342" s="42">
         <v>1</v>
       </c>
@@ -11470,7 +11470,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="343" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="343" spans="1:9" ht="34.15" thickBot="1" x14ac:dyDescent="0.85">
       <c r="A343" s="37">
         <v>2</v>
       </c>
@@ -11499,21 +11499,21 @@
         <v>6</v>
       </c>
     </row>
-    <row r="344" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="345" spans="1:9" ht="27" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A345" s="176" t="s">
+    <row r="344" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="345" spans="1:9" ht="25.15" thickBot="1" x14ac:dyDescent="0.95">
+      <c r="A345" s="179" t="s">
         <v>219</v>
       </c>
-      <c r="B345" s="177"/>
-      <c r="C345" s="177"/>
-      <c r="D345" s="177"/>
-      <c r="E345" s="177"/>
-      <c r="F345" s="177"/>
-      <c r="G345" s="177"/>
-      <c r="H345" s="177"/>
-      <c r="I345" s="178"/>
-    </row>
-    <row r="346" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B345" s="180"/>
+      <c r="C345" s="180"/>
+      <c r="D345" s="180"/>
+      <c r="E345" s="180"/>
+      <c r="F345" s="180"/>
+      <c r="G345" s="180"/>
+      <c r="H345" s="180"/>
+      <c r="I345" s="181"/>
+    </row>
+    <row r="346" spans="1:9" ht="21" thickBot="1" x14ac:dyDescent="0.8">
       <c r="A346" s="71" t="s">
         <v>38</v>
       </c>
@@ -11542,7 +11542,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="347" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="347" spans="1:9" ht="20.65" x14ac:dyDescent="0.75">
       <c r="A347" s="47">
         <v>3</v>
       </c>
@@ -11571,7 +11571,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="348" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="348" spans="1:9" ht="33.4" x14ac:dyDescent="0.75">
       <c r="A348" s="42">
         <v>5</v>
       </c>
@@ -11600,7 +11600,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="349" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="349" spans="1:9" ht="20.65" x14ac:dyDescent="0.75">
       <c r="A349" s="42">
         <v>2</v>
       </c>
@@ -11629,7 +11629,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="350" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="350" spans="1:9" ht="20.65" x14ac:dyDescent="0.75">
       <c r="A350" s="42">
         <v>6</v>
       </c>
@@ -11658,7 +11658,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="351" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="351" spans="1:9" ht="33.4" x14ac:dyDescent="0.75">
       <c r="A351" s="42">
         <v>1</v>
       </c>
@@ -11687,7 +11687,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="352" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="352" spans="1:9" ht="33.4" x14ac:dyDescent="0.75">
       <c r="A352" s="42">
         <v>4</v>
       </c>
@@ -11716,21 +11716,21 @@
         <v>6</v>
       </c>
     </row>
-    <row r="353" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="354" spans="1:9" ht="27" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A354" s="176" t="s">
+    <row r="353" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="354" spans="1:9" ht="25.15" thickBot="1" x14ac:dyDescent="0.95">
+      <c r="A354" s="179" t="s">
         <v>192</v>
       </c>
-      <c r="B354" s="177"/>
-      <c r="C354" s="177"/>
-      <c r="D354" s="177"/>
-      <c r="E354" s="177"/>
-      <c r="F354" s="177"/>
-      <c r="G354" s="177"/>
-      <c r="H354" s="177"/>
-      <c r="I354" s="178"/>
-    </row>
-    <row r="355" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B354" s="180"/>
+      <c r="C354" s="180"/>
+      <c r="D354" s="180"/>
+      <c r="E354" s="180"/>
+      <c r="F354" s="180"/>
+      <c r="G354" s="180"/>
+      <c r="H354" s="180"/>
+      <c r="I354" s="181"/>
+    </row>
+    <row r="355" spans="1:9" ht="21" thickBot="1" x14ac:dyDescent="0.8">
       <c r="A355" s="71" t="s">
         <v>38</v>
       </c>
@@ -11759,7 +11759,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="356" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="356" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A356" s="69">
         <v>4</v>
       </c>
@@ -11788,7 +11788,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="357" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="357" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A357" s="67">
         <v>3</v>
       </c>
@@ -11817,7 +11817,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="358" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="358" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A358" s="67">
         <v>5</v>
       </c>
@@ -11846,7 +11846,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="359" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="359" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A359" s="67">
         <v>2</v>
       </c>
@@ -11875,7 +11875,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="360" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="360" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A360" s="67">
         <v>1</v>
       </c>
@@ -11904,7 +11904,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="361" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="361" spans="1:9" ht="34.15" thickBot="1" x14ac:dyDescent="0.85">
       <c r="A361" s="61">
         <v>6</v>
       </c>
@@ -11933,21 +11933,21 @@
         <v>40</v>
       </c>
     </row>
-    <row r="362" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="363" spans="1:9" ht="27" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A363" s="176" t="s">
+    <row r="362" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="363" spans="1:9" ht="25.15" thickBot="1" x14ac:dyDescent="0.95">
+      <c r="A363" s="179" t="s">
         <v>162</v>
       </c>
-      <c r="B363" s="177"/>
-      <c r="C363" s="177"/>
-      <c r="D363" s="177"/>
-      <c r="E363" s="177"/>
-      <c r="F363" s="177"/>
-      <c r="G363" s="177"/>
-      <c r="H363" s="177"/>
-      <c r="I363" s="178"/>
-    </row>
-    <row r="364" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B363" s="180"/>
+      <c r="C363" s="180"/>
+      <c r="D363" s="180"/>
+      <c r="E363" s="180"/>
+      <c r="F363" s="180"/>
+      <c r="G363" s="180"/>
+      <c r="H363" s="180"/>
+      <c r="I363" s="181"/>
+    </row>
+    <row r="364" spans="1:9" ht="21" thickBot="1" x14ac:dyDescent="0.8">
       <c r="A364" s="71" t="s">
         <v>38</v>
       </c>
@@ -11976,7 +11976,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="365" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="365" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A365" s="69">
         <v>4</v>
       </c>
@@ -12005,7 +12005,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="366" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="366" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A366" s="67">
         <v>3</v>
       </c>
@@ -12034,7 +12034,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="367" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="367" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A367" s="67">
         <v>5</v>
       </c>
@@ -12063,7 +12063,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="368" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="368" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A368" s="67">
         <v>2</v>
       </c>
@@ -12092,7 +12092,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="369" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="369" spans="1:9" ht="29.25" x14ac:dyDescent="0.8">
       <c r="A369" s="67">
         <v>6</v>
       </c>
@@ -12121,7 +12121,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="370" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="370" spans="1:9" ht="34.15" thickBot="1" x14ac:dyDescent="0.85">
       <c r="A370" s="61">
         <v>1</v>
       </c>
@@ -12150,21 +12150,21 @@
         <v>6</v>
       </c>
     </row>
-    <row r="371" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="372" spans="1:9" ht="27" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A372" s="182" t="s">
+    <row r="371" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="372" spans="1:9" ht="25.15" thickBot="1" x14ac:dyDescent="0.95">
+      <c r="A372" s="184" t="s">
         <v>132</v>
       </c>
-      <c r="B372" s="183"/>
-      <c r="C372" s="183"/>
-      <c r="D372" s="183"/>
-      <c r="E372" s="183"/>
-      <c r="F372" s="183"/>
-      <c r="G372" s="183"/>
-      <c r="H372" s="183"/>
-      <c r="I372" s="184"/>
-    </row>
-    <row r="373" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B372" s="182"/>
+      <c r="C372" s="182"/>
+      <c r="D372" s="182"/>
+      <c r="E372" s="182"/>
+      <c r="F372" s="182"/>
+      <c r="G372" s="182"/>
+      <c r="H372" s="182"/>
+      <c r="I372" s="183"/>
+    </row>
+    <row r="373" spans="1:9" ht="21" thickBot="1" x14ac:dyDescent="0.8">
       <c r="A373" s="32" t="s">
         <v>38</v>
       </c>
@@ -12193,7 +12193,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="374" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="374" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A374" s="54">
         <v>4</v>
       </c>
@@ -12222,7 +12222,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="375" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="375" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A375" s="52">
         <v>5</v>
       </c>
@@ -12251,7 +12251,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="376" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="376" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A376" s="52">
         <v>3</v>
       </c>
@@ -12280,7 +12280,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="377" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="377" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A377" s="52">
         <v>2</v>
       </c>
@@ -12309,7 +12309,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="378" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="378" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A378" s="52">
         <v>1</v>
       </c>
@@ -12338,7 +12338,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="379" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="379" spans="1:9" ht="34.15" thickBot="1" x14ac:dyDescent="0.85">
       <c r="A379" s="49">
         <v>6</v>
       </c>
@@ -12367,21 +12367,21 @@
         <v>40</v>
       </c>
     </row>
-    <row r="380" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="381" spans="1:9" ht="27" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A381" s="176" t="s">
+    <row r="380" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="381" spans="1:9" ht="25.15" thickBot="1" x14ac:dyDescent="0.95">
+      <c r="A381" s="179" t="s">
         <v>101</v>
       </c>
-      <c r="B381" s="177"/>
-      <c r="C381" s="177"/>
-      <c r="D381" s="177"/>
-      <c r="E381" s="177"/>
-      <c r="F381" s="177"/>
-      <c r="G381" s="177"/>
-      <c r="H381" s="177"/>
-      <c r="I381" s="178"/>
-    </row>
-    <row r="382" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B381" s="180"/>
+      <c r="C381" s="180"/>
+      <c r="D381" s="180"/>
+      <c r="E381" s="180"/>
+      <c r="F381" s="180"/>
+      <c r="G381" s="180"/>
+      <c r="H381" s="180"/>
+      <c r="I381" s="181"/>
+    </row>
+    <row r="382" spans="1:9" ht="21" thickBot="1" x14ac:dyDescent="0.8">
       <c r="A382" s="32" t="s">
         <v>38</v>
       </c>
@@ -12410,7 +12410,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="383" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="383" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A383" s="54">
         <v>3</v>
       </c>
@@ -12439,7 +12439,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="384" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="384" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A384" s="52">
         <v>4</v>
       </c>
@@ -12468,7 +12468,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="385" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="385" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A385" s="52">
         <v>5</v>
       </c>
@@ -12497,7 +12497,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="386" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="386" spans="1:9" ht="21.4" x14ac:dyDescent="0.8">
       <c r="A386" s="52">
         <v>2</v>
       </c>
@@ -12526,7 +12526,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="387" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="387" spans="1:9" ht="33.75" x14ac:dyDescent="0.8">
       <c r="A387" s="52">
         <v>1</v>
       </c>
@@ -12555,7 +12555,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="388" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="388" spans="1:9" ht="34.15" thickBot="1" x14ac:dyDescent="0.85">
       <c r="A388" s="49">
         <v>6</v>
       </c>
@@ -12584,21 +12584,21 @@
         <v>6</v>
       </c>
     </row>
-    <row r="389" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="390" spans="1:9" ht="27" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A390" s="176" t="s">
+    <row r="389" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="390" spans="1:9" ht="25.15" thickBot="1" x14ac:dyDescent="0.95">
+      <c r="A390" s="179" t="s">
         <v>70</v>
       </c>
-      <c r="B390" s="177"/>
-      <c r="C390" s="177"/>
-      <c r="D390" s="177"/>
-      <c r="E390" s="177"/>
-      <c r="F390" s="177"/>
-      <c r="G390" s="177"/>
-      <c r="H390" s="177"/>
-      <c r="I390" s="178"/>
-    </row>
-    <row r="391" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B390" s="180"/>
+      <c r="C390" s="180"/>
+      <c r="D390" s="180"/>
+      <c r="E390" s="180"/>
+      <c r="F390" s="180"/>
+      <c r="G390" s="180"/>
+      <c r="H390" s="180"/>
+      <c r="I390" s="181"/>
+    </row>
+    <row r="391" spans="1:9" ht="21" thickBot="1" x14ac:dyDescent="0.8">
       <c r="A391" s="32" t="s">
         <v>38</v>
       </c>
@@ -12627,7 +12627,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="392" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="392" spans="1:9" ht="21.4" x14ac:dyDescent="0.8">
       <c r="A392" s="47">
         <v>4</v>
       </c>
@@ -12656,7 +12656,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="393" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="393" spans="1:9" ht="21.4" x14ac:dyDescent="0.8">
       <c r="A393" s="42">
         <v>3</v>
       </c>
@@ -12685,7 +12685,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="394" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="394" spans="1:9" ht="21.4" x14ac:dyDescent="0.8">
       <c r="A394" s="42">
         <v>5</v>
       </c>
@@ -12714,7 +12714,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="395" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="395" spans="1:9" ht="21.4" x14ac:dyDescent="0.8">
       <c r="A395" s="42">
         <v>6</v>
       </c>
@@ -12743,7 +12743,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="396" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+    <row r="396" spans="1:9" ht="21.4" x14ac:dyDescent="0.8">
       <c r="A396" s="42">
         <v>2</v>
       </c>
@@ -12772,7 +12772,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="397" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="397" spans="1:9" ht="21.75" thickBot="1" x14ac:dyDescent="0.85">
       <c r="A397" s="37">
         <v>1</v>
       </c>
@@ -12801,21 +12801,21 @@
         <v>40</v>
       </c>
     </row>
-    <row r="398" spans="1:9" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="399" spans="1:9" ht="27" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A399" s="176" t="s">
+    <row r="398" spans="1:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="399" spans="1:9" ht="25.15" thickBot="1" x14ac:dyDescent="0.95">
+      <c r="A399" s="179" t="s">
         <v>39</v>
       </c>
-      <c r="B399" s="177"/>
-      <c r="C399" s="177"/>
-      <c r="D399" s="177"/>
-      <c r="E399" s="177"/>
-      <c r="F399" s="177"/>
-      <c r="G399" s="177"/>
-      <c r="H399" s="177"/>
-      <c r="I399" s="178"/>
-    </row>
-    <row r="400" spans="1:9" ht="22" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B399" s="180"/>
+      <c r="C399" s="180"/>
+      <c r="D399" s="180"/>
+      <c r="E399" s="180"/>
+      <c r="F399" s="180"/>
+      <c r="G399" s="180"/>
+      <c r="H399" s="180"/>
+      <c r="I399" s="181"/>
+    </row>
+    <row r="400" spans="1:9" ht="21" thickBot="1" x14ac:dyDescent="0.8">
       <c r="A400" s="32" t="s">
         <v>38</v>
       </c>
@@ -12844,7 +12844,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="401" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+    <row r="401" spans="1:9" ht="33" x14ac:dyDescent="0.7">
       <c r="A401" s="26">
         <v>4</v>
       </c>
@@ -12873,7 +12873,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="402" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+    <row r="402" spans="1:9" ht="33" x14ac:dyDescent="0.7">
       <c r="A402" s="16">
         <v>6</v>
       </c>
@@ -12902,7 +12902,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="403" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+    <row r="403" spans="1:9" ht="33" x14ac:dyDescent="0.7">
       <c r="A403" s="16">
         <v>1</v>
       </c>
@@ -12931,7 +12931,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="404" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+    <row r="404" spans="1:9" ht="33" x14ac:dyDescent="0.7">
       <c r="A404" s="16">
         <v>2</v>
       </c>
@@ -12960,7 +12960,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="405" spans="1:9" ht="19" x14ac:dyDescent="0.25">
+    <row r="405" spans="1:9" ht="33" x14ac:dyDescent="0.7">
       <c r="A405" s="16">
         <v>3</v>
       </c>
@@ -12989,7 +12989,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="406" spans="1:9" ht="20" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="406" spans="1:9" ht="33.4" thickBot="1" x14ac:dyDescent="0.75">
       <c r="A406" s="8">
         <v>5</v>
       </c>
@@ -13020,41 +13020,6 @@
     </row>
   </sheetData>
   <mergeCells count="45">
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A10:I10"/>
-    <mergeCell ref="A19:I19"/>
-    <mergeCell ref="B28:I28"/>
-    <mergeCell ref="B37:I37"/>
-    <mergeCell ref="B46:I46"/>
-    <mergeCell ref="B55:I55"/>
-    <mergeCell ref="B65:I65"/>
-    <mergeCell ref="B75:I75"/>
-    <mergeCell ref="A84:I84"/>
-    <mergeCell ref="A93:I93"/>
-    <mergeCell ref="A102:I102"/>
-    <mergeCell ref="B111:I111"/>
-    <mergeCell ref="B120:I120"/>
-    <mergeCell ref="B129:I129"/>
-    <mergeCell ref="B138:I138"/>
-    <mergeCell ref="B147:I147"/>
-    <mergeCell ref="B156:I156"/>
-    <mergeCell ref="A165:I165"/>
-    <mergeCell ref="A174:I174"/>
-    <mergeCell ref="A183:I183"/>
-    <mergeCell ref="B192:I192"/>
-    <mergeCell ref="B201:I201"/>
-    <mergeCell ref="B210:I210"/>
-    <mergeCell ref="B219:I219"/>
-    <mergeCell ref="B228:I228"/>
-    <mergeCell ref="B237:I237"/>
-    <mergeCell ref="A246:I246"/>
-    <mergeCell ref="A255:I255"/>
-    <mergeCell ref="A264:I264"/>
-    <mergeCell ref="A273:I273"/>
-    <mergeCell ref="A282:I282"/>
-    <mergeCell ref="A291:I291"/>
-    <mergeCell ref="A300:I300"/>
-    <mergeCell ref="A309:I309"/>
     <mergeCell ref="A318:I318"/>
     <mergeCell ref="A381:I381"/>
     <mergeCell ref="A390:I390"/>
@@ -13065,6 +13030,41 @@
     <mergeCell ref="A354:I354"/>
     <mergeCell ref="A363:I363"/>
     <mergeCell ref="A372:I372"/>
+    <mergeCell ref="A273:I273"/>
+    <mergeCell ref="A282:I282"/>
+    <mergeCell ref="A291:I291"/>
+    <mergeCell ref="A300:I300"/>
+    <mergeCell ref="A309:I309"/>
+    <mergeCell ref="B228:I228"/>
+    <mergeCell ref="B237:I237"/>
+    <mergeCell ref="A246:I246"/>
+    <mergeCell ref="A255:I255"/>
+    <mergeCell ref="A264:I264"/>
+    <mergeCell ref="A183:I183"/>
+    <mergeCell ref="B192:I192"/>
+    <mergeCell ref="B201:I201"/>
+    <mergeCell ref="B210:I210"/>
+    <mergeCell ref="B219:I219"/>
+    <mergeCell ref="B138:I138"/>
+    <mergeCell ref="B147:I147"/>
+    <mergeCell ref="B156:I156"/>
+    <mergeCell ref="A165:I165"/>
+    <mergeCell ref="A174:I174"/>
+    <mergeCell ref="A93:I93"/>
+    <mergeCell ref="A102:I102"/>
+    <mergeCell ref="B111:I111"/>
+    <mergeCell ref="B120:I120"/>
+    <mergeCell ref="B129:I129"/>
+    <mergeCell ref="B46:I46"/>
+    <mergeCell ref="B55:I55"/>
+    <mergeCell ref="B65:I65"/>
+    <mergeCell ref="B75:I75"/>
+    <mergeCell ref="A84:I84"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A10:I10"/>
+    <mergeCell ref="A19:I19"/>
+    <mergeCell ref="B28:I28"/>
+    <mergeCell ref="B37:I37"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="72" fitToHeight="0" orientation="portrait" r:id="rId1"/>

</xml_diff>